<commit_message>
feat: complete stage two data governance
</commit_message>
<xml_diff>
--- a/outputs/aapl_market_signal.xlsx
+++ b/outputs/aapl_market_signal.xlsx
@@ -8,15 +8,25 @@
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="行情数据" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="新闻舆情" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="数据质量" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="主体信息" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="行情数据" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="财务数据" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="新闻舆情" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="公告数据" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="指标分析" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="数据来源" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="数据质量" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$C$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'行情数据'!$A$1:$G$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'新闻舆情'!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'数据质量'!$A$1:$D$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$C$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'主体信息'!$A$1:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'行情数据'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'财务数据'!$A$1:$L$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'新闻舆情'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'公告数据'!$A$1:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'指标分析'!$A$1:$F$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'数据来源'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'数据质量'!$A$1:$D$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -73,7 +83,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -85,6 +95,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -454,12 +467,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="47" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,166 +505,343 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Single-stock stage-one run</t>
+          <t>Single-stock stage-two run</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>start_date</t>
+          <t>company_name</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>Apple Inc.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Inclusive request boundary</t>
+          <t>Resolved from SEC entity data</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>end_date</t>
+          <t>cik</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>0000320193</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Inclusive request boundary</t>
+          <t>SEC central index key</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>mode</t>
+          <t>exchange</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>fixture</t>
+          <t>Nasdaq</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>fixture is deterministic; online uses source adapters</t>
+          <t>Resolved from SEC entity data</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>price_source</t>
+          <t>start_date</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>fixture:/Users/yinjuanxi/Downloads/AAA水水大王/fixtures/aapl_prices.json</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Source URL or fixture path</t>
+          <t>Inclusive market/news/filing boundary</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>news_source</t>
+          <t>end_date</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>fixture:/Users/yinjuanxi/Downloads/AAA水水大王/fixtures/aapl_news.xml</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Source URL or fixture path</t>
+          <t>Inclusive market/news/filing boundary</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>price_rows</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>5</v>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Rows after cleaning</t>
+          <t>fixture is deterministic; online uses source adapters</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>news_rows</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>2</v>
+          <t>pipeline_status</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Rows after cleaning</t>
+          <t>Review 数据质量 and 数据来源 for details</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>forecast_status</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>not implemented in stage one</t>
-        </is>
+          <t>price_rows</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Forecasting is planned for a later stage</t>
+          <t>Rows after cleaning and range filtering</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>financial_rows</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Rows after cleaning and availability filtering</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>news_rows</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Rows after cleaning and range filtering</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>announcement_rows</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Rows after cleaning and range filtering</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>indicator_rows</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Derived market, financial, news, and filing indicators</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>forecast_status</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>not implemented in stage two</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Forecasting is planned for a later stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>limitations</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Financial statements and sentiment scoring are not included</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Do not treat this workbook as investment advice</t>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Rule-based news tone is not investment advice</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Financial data is limited to configured SEC concepts</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C11"/>
+  <autoFilter ref="A1:C16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>symbol</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>company_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>cik</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>exchange</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>sic</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>sic_description</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0000320193</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>3571</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Electronic Computers</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>fixture:SEC entity data</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -666,7 +856,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -729,7 +919,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>fixture:/Users/yinjuanxi/Downloads/AAA水水大王/fixtures/aapl_prices.json</t>
+          <t>fixture:prices</t>
         </is>
       </c>
     </row>
@@ -756,7 +946,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>fixture:/Users/yinjuanxi/Downloads/AAA水水大王/fixtures/aapl_prices.json</t>
+          <t>fixture:prices</t>
         </is>
       </c>
     </row>
@@ -783,7 +973,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>fixture:/Users/yinjuanxi/Downloads/AAA水水大王/fixtures/aapl_prices.json</t>
+          <t>fixture:prices</t>
         </is>
       </c>
     </row>
@@ -810,7 +1000,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>fixture:/Users/yinjuanxi/Downloads/AAA水水大王/fixtures/aapl_prices.json</t>
+          <t>fixture:prices</t>
         </is>
       </c>
     </row>
@@ -837,135 +1027,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>fixture:/Users/yinjuanxi/Downloads/AAA水水大王/fixtures/aapl_prices.json</t>
+          <t>fixture:prices</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G6"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>published_at</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>summary</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>sentiment</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Thu, 13 Aug 2026 13:30:00 GMT</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Apple shares close after product update</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Example Markets</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>https://example.com/aapl/product-update</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Second fixture article.</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>unclassified</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Fri, 14 Aug 2026 14:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Apple supplier update highlights demand outlook</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Example Finance</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>https://example.com/aapl/supplier-update</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Fixture article retained for deterministic stage-one validation.</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>unclassified</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F3"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -976,40 +1043,1715 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="47" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>period_start</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>period_end</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>filed_date</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>fiscal_year</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>fiscal_period</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>form</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>metric</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>metric_label</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>notes</t>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>accession_number</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>net_income</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Net income</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>23000000000</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>0000320193-26-000002</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>fixture:SEC companyfacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>88000000000</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>0000320193-26-000002</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>fixture:SEC companyfacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>assets</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Total assets</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>364000000000</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>0000320193-26-000003</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>fixture:SEC companyfacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>cash_and_equivalents</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>35000000000</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>0000320193-26-000003</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>fixture:SEC companyfacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>current_assets</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Current assets</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>124000000000</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>0000320193-26-000003</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>fixture:SEC companyfacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>current_liabilities</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Current liabilities</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>131000000000</v>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>0000320193-26-000003</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>fixture:SEC companyfacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>liabilities</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Total liabilities</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>282000000000</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>0000320193-26-000003</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>fixture:SEC companyfacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>net_income</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Net income</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>24500000000</v>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>0000320193-26-000003</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>fixture:SEC companyfacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>operating_cash_flow</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Operating cash flow</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>28000000000</v>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>0000320193-26-000003</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>fixture:SEC companyfacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>94000000000</v>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>0000320193-26-000003</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>fixture:SEC companyfacts</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="49" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>published_at</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>sentiment</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>sentiment_basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 13:30:00 GMT</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Apple shares close after product update</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Example Markets</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>https://example.com/aapl/product-update</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Second fixture article.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>no configured keyword matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Fri, 14 Aug 2026 14:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Apple supplier update highlights demand outlook</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Example Finance</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>https://example.com/aapl/supplier-update</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Fixture article retained for deterministic stage-two validation.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>demand</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G3"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>filed_date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>report_date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>form</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>accession_number</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>8-K</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Current report</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>0000320193-26-000004</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/320193/000032019326000004/aapl-20260814.htm</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>fixture:SEC submissions</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G2"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>indicator</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>latest_close</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>305.93</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>last clean close</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>period_return</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>-0.7558554467008318</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>(last close / first close - 1) * 100</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10 to 2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>average_close</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>305.322</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>mean of clean closes</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>5 records</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>average_volume</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>38505140</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>shares</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>mean of clean volumes</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>5 records</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>close_return_volatility</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.8431625272924098</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>population standard deviation of close-to-close returns</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>4 return observations</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>positive_news_count</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>rule-based keyword classification</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>title and summary retained in 新闻舆情</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>negative_news_count</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>rule-based keyword classification</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>title and summary retained in 新闻舆情</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>neutral_news_count</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>rule-based keyword classification</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>title and summary retained in 新闻舆情</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>news_tone_balance</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>positive count minus negative count</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>rule-based keyword classification</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>filing_count</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>filings</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>count of clean SEC filings</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>10-K, 10-Q, and 8-K only</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>financial</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>net_profit_margin</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>26.06382978723405</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>net income / revenue * 100 for the same reporting period</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01 to 2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>financial</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>current_ratio</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>0.9465648854961832</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>current assets / current liabilities at the same period end</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>financial</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>operating_cash_flow_margin</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>29.78723404255319</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>operating cash flow / revenue * 100 for the same reporting period</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01 to 2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>financial</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>revenue_period_change</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>6.818181818181817</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>(latest revenue / prior comparable-duration revenue - 1) * 100</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01 to 2026-03-31 compared with 2026-04-01 to 2026-06-30</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>provider</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>cache_status</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>source_location</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>raw_rows</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>clean_rows</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>output_rows</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>prices</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>loaded</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>fixture:fixtures/aapl_prices.json</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>daily OHLCV data</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>loaded</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>fixture:fixtures/aapl_news.xml</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>news headlines and source text</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>entity</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>loaded</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>fixture:fixtures/aapl_entity.json</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>symbol-to-CIK mapping and entity attributes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>financials</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>loaded</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>fixture:fixtures/aapl_financials.json</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>configured US-GAAP concepts from 10-K and 10-Q filings</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>loaded</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>fixture:fixtures/aapl_submissions.json</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>10-K, 10-Q, and 8-K filing history</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>prices</t>
         </is>
       </c>
@@ -1023,7 +2765,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>rows received from source</t>
+          <t>processing quality metric</t>
         </is>
       </c>
     </row>
@@ -1043,7 +2785,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>rows written to workbook</t>
+          <t>processing quality metric</t>
         </is>
       </c>
     </row>
@@ -1055,15 +2797,15 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>duplicates_removed</t>
+          <t>output_rows</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>duplicate dates removed</t>
+          <t>processing quality metric</t>
         </is>
       </c>
     </row>
@@ -1075,7 +2817,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>invalid_rows</t>
+          <t>duplicates_removed</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -1083,7 +2825,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>invalid rows discarded</t>
+          <t>processing quality metric</t>
         </is>
       </c>
     </row>
@@ -1095,107 +2837,107 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>out_of_range</t>
+          <t>invalid_rows</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>rows outside request boundaries</t>
+          <t>processing quality metric</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>prices</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>raw_rows</t>
+          <t>out_of_range</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>rows received from source</t>
+          <t>processing quality metric</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>financials</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>clean_rows</t>
+          <t>raw_rows</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>rows written to workbook</t>
+          <t>processing quality metric</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>financials</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>duplicates_removed</t>
+          <t>clean_rows</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>duplicate records removed</t>
+          <t>processing quality metric</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>financials</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>invalid_rows</t>
+          <t>output_rows</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>invalid rows discarded</t>
+          <t>processing quality metric</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>financials</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>out_of_range</t>
+          <t>duplicates_removed</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1203,34 +2945,314 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>rows outside request boundaries</t>
+          <t>processing quality metric</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>financials</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>invalid_rows</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>financials</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>out_of_range</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>raw_rows</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>clean_rows</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>output_rows</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>duplicates_removed</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>invalid_rows</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>out_of_range</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>raw_rows</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>clean_rows</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>output_rows</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>duplicates_removed</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>invalid_rows</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>out_of_range</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>processing quality metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>pipeline</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>warning means a source returned no clean rows</t>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>warning means one or more required datasets have no clean rows</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D12"/>
+  <autoFilter ref="A1:D26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: support Chinese stock markets
</commit_message>
<xml_diff>
--- a/outputs/aapl_market_signal.xlsx
+++ b/outputs/aapl_market_signal.xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="主体信息" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="行情数据" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="财务数据" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="新闻舆情" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="公告数据" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="指标分析" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="数据来源" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="数据质量" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主体信息" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行情数据" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="财务数据" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新闻舆情" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="公告数据" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标分析" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据来源" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据质量" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$C$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'主体信息'!$A$1:$G$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'行情数据'!$A$1:$G$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'财务数据'!$A$1:$L$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'新闻舆情'!$A$1:$G$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'公告数据'!$A$1:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$C$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'主体信息'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'行情数据'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'财务数据'!$A$1:$N$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'新闻舆情'!$A$1:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'公告数据'!$A$1:$I$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'指标分析'!$A$1:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'数据来源'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'数据来源'!$A$1:$L$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'数据质量'!$A$1:$D$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -505,7 +505,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Single-stock stage-two run</t>
+          <t>Single-stock multi-market run</t>
         </is>
       </c>
     </row>
@@ -522,165 +522,171 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Resolved from SEC entity data</t>
+          <t>Resolved from the selected market data source</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>cik</t>
+          <t>provider_symbol</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>0000320193</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>SEC central index key</t>
+          <t>Symbol passed to the selected data source</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>exchange</t>
+          <t>market</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Nasdaq</t>
+          <t>us</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Resolved from SEC entity data</t>
+          <t>美国股票</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>start_date</t>
+          <t>cik</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>0000320193</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Inclusive market/news/filing boundary</t>
+          <t>SEC central index key when available</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>end_date</t>
+          <t>exchange</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>Nasdaq</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Inclusive market/news/filing boundary</t>
+          <t>Resolved from the selected market data source</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>mode</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>fixture</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>fixture is deterministic; online uses source adapters</t>
+          <t>Reporting currency from market or source</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>pipeline_status</t>
+          <t>start_date</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Review 数据质量 and 数据来源 for details</t>
+          <t>Inclusive market/news/filing boundary</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>price_rows</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>5</v>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Rows after cleaning and range filtering</t>
+          <t>Inclusive market/news/filing boundary</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>financial_rows</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>10</v>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Rows after cleaning and availability filtering</t>
+          <t>fixture is deterministic; online uses source adapters</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>news_rows</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>2</v>
+          <t>pipeline_status</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Rows after cleaning and range filtering</t>
+          <t>Review 数据质量 and 数据来源 for details</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>announcement_rows</t>
+          <t>price_rows</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
@@ -691,54 +697,99 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>indicator_rows</t>
+          <t>financial_rows</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Derived market, financial, news, and filing indicators</t>
+          <t>Rows after cleaning and availability filtering</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>forecast_status</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>not implemented in stage two</t>
-        </is>
+          <t>news_rows</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Forecasting is planned for a later stage</t>
+          <t>Rows after cleaning and range filtering</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>announcement_rows</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Rows after cleaning and range filtering</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>indicator_rows</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Derived market, financial, news, and filing indicators</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>forecast_status</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>not implemented in stage two</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Forecasting is planned for a later stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>limitations</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Rule-based news tone is not investment advice</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Financial data is limited to configured SEC concepts</t>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Financial coverage varies by market adapter</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C16"/>
+  <autoFilter ref="A1:C19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -749,16 +800,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -774,25 +829,45 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>provider_symbol</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>market_name</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>cik</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>exchange</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>sic</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>sic_description</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
@@ -811,32 +886,52 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>美国股票</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>0000320193</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Nasdaq</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>3571</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Electronic Computers</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>fixture:SEC entity data</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G2"/>
+  <autoFilter ref="A1:K2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -847,7 +942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -857,6 +952,8 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -895,6 +992,16 @@
           <t>source</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -922,6 +1029,16 @@
           <t>fixture:prices</t>
         </is>
       </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -949,6 +1066,16 @@
           <t>fixture:prices</t>
         </is>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -976,6 +1103,16 @@
           <t>fixture:prices</t>
         </is>
       </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1003,6 +1140,16 @@
           <t>fixture:prices</t>
         </is>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1030,9 +1177,19 @@
           <t>fixture:prices</t>
         </is>
       </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G6"/>
+  <autoFilter ref="A1:I6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1043,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1058,6 +1215,8 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
     <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1121,6 +1280,16 @@
           <t>source</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1179,6 +1348,16 @@
           <t>fixture:SEC companyfacts</t>
         </is>
       </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1235,6 +1414,16 @@
       <c r="L3" s="2" t="inlineStr">
         <is>
           <t>fixture:SEC companyfacts</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
         </is>
       </c>
     </row>
@@ -1291,6 +1480,16 @@
           <t>fixture:SEC companyfacts</t>
         </is>
       </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr"/>
@@ -1345,6 +1544,16 @@
           <t>fixture:SEC companyfacts</t>
         </is>
       </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr"/>
@@ -1399,6 +1608,16 @@
           <t>fixture:SEC companyfacts</t>
         </is>
       </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr"/>
@@ -1453,6 +1672,16 @@
           <t>fixture:SEC companyfacts</t>
         </is>
       </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr"/>
@@ -1507,6 +1736,16 @@
           <t>fixture:SEC companyfacts</t>
         </is>
       </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1565,6 +1804,16 @@
           <t>fixture:SEC companyfacts</t>
         </is>
       </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1623,6 +1872,16 @@
           <t>fixture:SEC companyfacts</t>
         </is>
       </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1681,9 +1940,19 @@
           <t>fixture:SEC companyfacts</t>
         </is>
       </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L11"/>
+  <autoFilter ref="A1:N11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1694,7 +1963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -1704,6 +1973,8 @@
     <col width="52" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="31" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1742,6 +2013,16 @@
           <t>sentiment_basis</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1779,6 +2060,16 @@
           <t>no configured keyword matched</t>
         </is>
       </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1816,9 +2107,19 @@
           <t>demand</t>
         </is>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:I3"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -1833,7 +2134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1843,6 +2144,8 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1881,6 +2184,16 @@
           <t>source</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1918,9 +2231,19 @@
           <t>fixture:SEC submissions</t>
         </is>
       </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G2"/>
+  <autoFilter ref="A1:I2"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
   </hyperlinks>
@@ -2268,12 +2591,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>count of clean SEC filings</t>
+          <t>count of clean market notices and filings</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>10-K, 10-Q, and 8-K only</t>
+          <t>clean announcement and filing rows</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2421,7 +2744,9 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2475,6 +2800,16 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2521,6 +2856,16 @@
           <t>daily OHLCV data</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2567,6 +2912,16 @@
           <t>news headlines and source text</t>
         </is>
       </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2610,7 +2965,17 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>symbol-to-CIK mapping and entity attributes</t>
+          <t>symbol-to-entity mapping and entity attributes</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
         </is>
       </c>
     </row>
@@ -2656,7 +3021,17 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>configured US-GAAP concepts from 10-K and 10-Q filings</t>
+          <t>configured fixture financial concepts</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
         </is>
       </c>
     </row>
@@ -2702,12 +3077,22 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>10-K, 10-Q, and 8-K filing history</t>
+          <t>market filing and notice history</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:L6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: complete real-data forecasting stage
</commit_message>
<xml_diff>
--- a/outputs/aapl_market_signal.xlsx
+++ b/outputs/aapl_market_signal.xlsx
@@ -762,12 +762,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>not implemented in stage two</t>
+          <t>not requested</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Forecasting is planned for a later stage</t>
+          <t>Forecasting requires online stage-two data</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: complete scalable operations stage
</commit_message>
<xml_diff>
--- a/outputs/aapl_market_signal.xlsx
+++ b/outputs/aapl_market_signal.xlsx
@@ -16,9 +16,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标分析" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据来源" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据质量" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本信息" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$C$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$C$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'主体信息'!$A$1:$K$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'行情数据'!$A$1:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'财务数据'!$A$1:$N$11</definedName>
@@ -27,6 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'指标分析'!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'数据来源'!$A$1:$L$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'数据质量'!$A$1:$D$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'版本信息'!$A$1:$C$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -467,10 +469,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="47" customWidth="1" min="2" max="2"/>
     <col width="52" customWidth="1" min="3" max="3"/>
   </cols>
@@ -774,22 +776,348 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>cross_validation_status</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>not requested</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Optional secondary-source close comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>limitations</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Rule-based news tone is not investment advice</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Financial coverage varies by market adapter</t>
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>version_skill</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Central component version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>version_data_contract</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Central component version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>version_batch_contract</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Central component version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>version_source_adapters</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Central component version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>version_forecast_engine</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Central component version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>version_workbook_template</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Central component version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>version_last_close_baseline</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>persistence-v1</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Central component version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>version_multisignal_ridge</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>ridge-v1</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Central component version registry</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C19"/>
+  <autoFilter ref="A1:C28"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>central version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>data_contract</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>central version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>batch_contract</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>central version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>source_adapters</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>central version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>forecast_engine</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>central version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>workbook_template</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>central version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>last_close_baseline</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>persistence-v1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>central version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>multisignal_ridge</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>ridge-v1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>central version registry</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: improve forecast model selection
</commit_message>
<xml_diff>
--- a/outputs/aapl_market_signal.xlsx
+++ b/outputs/aapl_market_signal.xlsx
@@ -19,7 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本信息" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$C$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$C$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'主体信息'!$A$1:$K$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'行情数据'!$A$1:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'财务数据'!$A$1:$N$11</definedName>
@@ -28,7 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'指标分析'!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'数据来源'!$A$1:$L$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'数据质量'!$A$1:$D$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'版本信息'!$A$1:$C$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'版本信息'!$A$1:$C$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,10 +469,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="47" customWidth="1" min="2" max="2"/>
     <col width="52" customWidth="1" min="3" max="3"/>
   </cols>
@@ -815,7 +815,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -929,22 +929,73 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>version_moving_average_baseline</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>moving-average-v1</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Central component version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>version_historical_mean_baseline</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>historical-mean-v1</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Central component version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>version_exponential_smoothing_baseline</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>ewma-v1</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Central component version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>version_multisignal_ridge</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>ridge-v1</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Central component version registry</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C28"/>
+  <autoFilter ref="A1:C31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -955,11 +1006,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -988,7 +1039,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1005,7 +1056,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1022,7 +1073,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1056,7 +1107,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1073,7 +1124,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1102,22 +1153,73 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>moving_average_baseline</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>moving-average-v1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>central version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>historical_mean_baseline</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>historical-mean-v1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>central version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>exponential_smoothing_baseline</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ewma-v1</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>central version registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>multisignal_ridge</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>ridge-v1</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>central version registry</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C9"/>
+  <autoFilter ref="A1:C12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>